<commit_message>
Update all pending changes: dashboard, templates, docs, DB schema
- Update dashboard.py with business KPI improvements
- Update CI/PI/OC/PL templates for cell position fixes
- Add dashboard guide, data join guide, data pipeline vision docs
- Update DB schema, config, utils, excel generator
- Add dashboard tests and order_book.xlsx
- Update .gitignore to exclude dashboard_dist/ and test_output.txt

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/order_confirmation.xlsx
+++ b/templates/order_confirmation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FB823D1-F586-4546-AF6B-A2A1D8E2441B}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED9A1991-290A-4EB2-9FE7-3F6D99A230FA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9590" yWindow="-21710" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -72,9 +72,6 @@
     <t>EA</t>
   </si>
   <si>
-    <t>USD</t>
-  </si>
-  <si>
     <t>Full General Sales Terms Conditions can be found at</t>
   </si>
   <si>
@@ -126,6 +123,10 @@
   </si>
   <si>
     <t>Date:</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>USD</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
 </sst>
@@ -139,7 +140,7 @@
     <numFmt numFmtId="177" formatCode="#,##0.00_ "/>
     <numFmt numFmtId="178" formatCode="#,##0.00_);[Red]\(#,##0.00\)"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -311,6 +312,13 @@
       <b/>
       <sz val="8.5"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -508,9 +516,6 @@
     <xf numFmtId="1" fontId="17" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="3" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -558,48 +563,9 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="176" fontId="17" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -610,24 +576,66 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+      <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="17" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -668,7 +676,7 @@
       <xdr:col>8</xdr:col>
       <xdr:colOff>727387</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>89167</xdr:rowOff>
+      <xdr:rowOff>92342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1007,17 +1015,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="58" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
+      <c r="A1" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -1033,13 +1041,13 @@
       <c r="J2" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1047,13 +1055,13 @@
       <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1061,13 +1069,13 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -1087,35 +1095,35 @@
       <c r="J6" s="13"/>
     </row>
     <row r="7" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="49"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="13"/>
+    </row>
+    <row r="8" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="64"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="62"/>
-      <c r="E7" s="62"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="24" t="s">
+      <c r="B8" s="50"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="62"/>
-      <c r="I7" s="62"/>
-      <c r="J7" s="13"/>
-    </row>
-    <row r="8" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="65" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="65"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
       <c r="J8" s="13"/>
     </row>
     <row r="9" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1125,11 +1133,11 @@
       <c r="D9" s="19"/>
       <c r="E9" s="19"/>
       <c r="F9" s="20"/>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
       <c r="J9" s="13"/>
     </row>
     <row r="10" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1139,11 +1147,11 @@
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="20"/>
-      <c r="G10" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
+      <c r="G10" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
       <c r="J10" s="13"/>
     </row>
     <row r="11" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1153,68 +1161,68 @@
       <c r="D11" s="19"/>
       <c r="E11" s="19"/>
       <c r="F11" s="20"/>
-      <c r="G11" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="H11" s="54"/>
-      <c r="I11" s="54"/>
+      <c r="G11" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="51"/>
+      <c r="I11" s="51"/>
       <c r="J11" s="13"/>
     </row>
     <row r="12" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
-        <v>17</v>
+      <c r="A12" s="22" t="s">
+        <v>16</v>
       </c>
       <c r="E12" s="17"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="54"/>
+      <c r="I12" s="54"/>
       <c r="J12" s="13"/>
     </row>
     <row r="13" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="54"/>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
+      <c r="A13" s="51"/>
+      <c r="B13" s="51"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="51"/>
+      <c r="E13" s="51"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="51"/>
       <c r="J13" s="13"/>
     </row>
     <row r="14" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="54"/>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
+      <c r="A14" s="51"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="51"/>
+      <c r="E14" s="51"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="G14" s="51"/>
+      <c r="H14" s="51"/>
+      <c r="I14" s="51"/>
       <c r="J14" s="13"/>
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="54"/>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
+      <c r="A15" s="51"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
       <c r="F15" s="15"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="51"/>
       <c r="J15" s="13"/>
     </row>
     <row r="16" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
+      <c r="B16" s="56"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
       <c r="F16" s="15"/>
       <c r="G16" s="19"/>
       <c r="H16" s="15"/>
@@ -1222,147 +1230,147 @@
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="66" t="s">
+      <c r="A17" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="67"/>
-      <c r="C17" s="67"/>
-      <c r="D17" s="67"/>
-      <c r="E17" s="27" t="s">
+      <c r="B17" s="53"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="H17" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" s="29" t="s">
+      <c r="H17" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" s="28" t="s">
         <v>8</v>
       </c>
       <c r="J17" s="13"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="44"/>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="34"/>
+      <c r="A18" s="47"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="33"/>
       <c r="I18" s="68"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="44"/>
-      <c r="B19" s="45"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="34"/>
+      <c r="A19" s="47"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="33"/>
       <c r="I19" s="68"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="44"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="34"/>
+      <c r="A20" s="47"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="33"/>
       <c r="I20" s="68"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="44"/>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="A21" s="47"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="33"/>
       <c r="I21" s="68"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="44"/>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="34"/>
+      <c r="A22" s="47"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="33"/>
       <c r="I22" s="68"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="44"/>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="34"/>
+      <c r="A23" s="47"/>
+      <c r="B23" s="48"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="33"/>
       <c r="I23" s="68"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="42"/>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="36"/>
+      <c r="A24" s="58"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="35"/>
       <c r="I24" s="69"/>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="52" t="s">
+      <c r="A25" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="53"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="53"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
       <c r="E25" s="21">
         <f>SUM(E18:E24)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="39" t="s">
+      <c r="F25" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="G25" s="22"/>
-      <c r="H25" s="39" t="s">
-        <v>11</v>
-      </c>
-      <c r="I25" s="70">
+      <c r="G25" s="70" t="s">
+        <v>24</v>
+      </c>
+      <c r="H25" s="38"/>
+      <c r="I25" s="39">
         <f>SUM(I18:I24)</f>
         <v>0</v>
       </c>
       <c r="J25" s="2"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="50"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="51"/>
-      <c r="E26" s="51"/>
-      <c r="F26" s="51"/>
-      <c r="G26" s="51"/>
-      <c r="H26" s="51"/>
-      <c r="I26" s="51"/>
+      <c r="A26" s="64"/>
+      <c r="B26" s="65"/>
+      <c r="C26" s="65"/>
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
+      <c r="I26" s="65"/>
       <c r="J26" s="3"/>
     </row>
     <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1529,49 +1537,65 @@
       <c r="J40" s="6"/>
     </row>
     <row r="41" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="48" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="49"/>
-      <c r="C41" s="49"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="49"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
-      <c r="I41" s="49"/>
+      <c r="A41" s="62" t="s">
+        <v>17</v>
+      </c>
+      <c r="B41" s="63"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="63"/>
+      <c r="I41" s="63"/>
       <c r="J41" s="6"/>
     </row>
     <row r="42" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="25"/>
-      <c r="B42" s="26"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="25"/>
       <c r="J42" s="6"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" s="46" t="s">
+      <c r="A43" s="60" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" s="61"/>
+      <c r="C43" s="61"/>
+      <c r="D43" s="61"/>
+      <c r="E43" s="61"/>
+      <c r="F43" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="47"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="47"/>
-      <c r="F43" s="56" t="s">
-        <v>13</v>
-      </c>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="46"/>
+      <c r="I43" s="46"/>
       <c r="J43" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="G13:I15"/>
+    <mergeCell ref="F43:I43"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="H7:I7"/>
@@ -1588,22 +1612,6 @@
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="G13:I15"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Fix OC Total row Currency column: H → G to match item rows
The Total row was writing Currency to H column (hardcoded) while item rows
used COL_CURRENCY = 'G'. Now uses the COL_CURRENCY constant consistently.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/order_confirmation.xlsx
+++ b/templates/order_confirmation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED9A1991-290A-4EB2-9FE7-3F6D99A230FA}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFD3E7B3-37C5-415B-955F-3584A1484247}"/>
   <bookViews>
-    <workbookView xWindow="-9590" yWindow="-21710" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Rotork Controls Korea Co., Ltd.</t>
   </si>
@@ -123,10 +123,6 @@
   </si>
   <si>
     <t>Date:</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>USD</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
 </sst>
@@ -566,6 +562,57 @@
     <xf numFmtId="176" fontId="17" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -576,67 +623,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
@@ -1015,17 +1011,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
       <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -1041,13 +1037,13 @@
       <c r="J2" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1055,13 +1051,13 @@
       <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
+      <c r="B4" s="60"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1069,13 +1065,13 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -1095,35 +1091,35 @@
       <c r="J6" s="13"/>
     </row>
     <row r="7" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
+      <c r="B7" s="67"/>
+      <c r="C7" s="65"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
       <c r="F7" s="20"/>
       <c r="G7" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="44"/>
-      <c r="I7" s="44"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="65"/>
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="50"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
+      <c r="B8" s="68"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
       <c r="F8" s="20"/>
       <c r="G8" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="51"/>
-      <c r="I8" s="51"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="57"/>
       <c r="J8" s="13"/>
     </row>
     <row r="9" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1136,8 +1132,8 @@
       <c r="G9" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="57"/>
       <c r="J9" s="13"/>
     </row>
     <row r="10" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1150,8 +1146,8 @@
       <c r="G10" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="51"/>
-      <c r="I10" s="51"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="57"/>
       <c r="J10" s="13"/>
     </row>
     <row r="11" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1164,8 +1160,8 @@
       <c r="G11" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="51"/>
-      <c r="I11" s="51"/>
+      <c r="H11" s="57"/>
+      <c r="I11" s="57"/>
       <c r="J11" s="13"/>
     </row>
     <row r="12" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1177,52 +1173,52 @@
       <c r="G12" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="54"/>
-      <c r="I12" s="54"/>
+      <c r="H12" s="58"/>
+      <c r="I12" s="58"/>
       <c r="J12" s="13"/>
     </row>
     <row r="13" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="51"/>
-      <c r="B13" s="51"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
+      <c r="A13" s="57"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="57"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="51"/>
-      <c r="H13" s="51"/>
-      <c r="I13" s="51"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="57"/>
+      <c r="I13" s="57"/>
       <c r="J13" s="13"/>
     </row>
     <row r="14" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="51"/>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
+      <c r="A14" s="57"/>
+      <c r="B14" s="57"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="51"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="51"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
+      <c r="I14" s="57"/>
       <c r="J14" s="13"/>
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="51"/>
-      <c r="B15" s="51"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="51"/>
+      <c r="A15" s="57"/>
+      <c r="B15" s="57"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="57"/>
       <c r="F15" s="15"/>
-      <c r="G15" s="51"/>
-      <c r="H15" s="51"/>
-      <c r="I15" s="51"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="57"/>
       <c r="J15" s="13"/>
     </row>
     <row r="16" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
-      <c r="B16" s="56"/>
-      <c r="C16" s="57"/>
-      <c r="D16" s="57"/>
-      <c r="E16" s="57"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
       <c r="F16" s="15"/>
       <c r="G16" s="19"/>
       <c r="H16" s="15"/>
@@ -1230,12 +1226,12 @@
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="70"/>
       <c r="E17" s="26" t="s">
         <v>5</v>
       </c>
@@ -1262,7 +1258,7 @@
       <c r="F18" s="36"/>
       <c r="G18" s="32"/>
       <c r="H18" s="33"/>
-      <c r="I18" s="68"/>
+      <c r="I18" s="40"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1274,7 +1270,7 @@
       <c r="F19" s="36"/>
       <c r="G19" s="32"/>
       <c r="H19" s="33"/>
-      <c r="I19" s="68"/>
+      <c r="I19" s="40"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1286,7 +1282,7 @@
       <c r="F20" s="36"/>
       <c r="G20" s="32"/>
       <c r="H20" s="33"/>
-      <c r="I20" s="68"/>
+      <c r="I20" s="40"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1298,7 +1294,7 @@
       <c r="F21" s="36"/>
       <c r="G21" s="32"/>
       <c r="H21" s="33"/>
-      <c r="I21" s="68"/>
+      <c r="I21" s="40"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1310,7 +1306,7 @@
       <c r="F22" s="36"/>
       <c r="G22" s="32"/>
       <c r="H22" s="33"/>
-      <c r="I22" s="68"/>
+      <c r="I22" s="40"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1322,28 +1318,28 @@
       <c r="F23" s="36"/>
       <c r="G23" s="32"/>
       <c r="H23" s="33"/>
-      <c r="I23" s="68"/>
+      <c r="I23" s="40"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="58"/>
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="59"/>
+      <c r="A24" s="45"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
       <c r="E24" s="31"/>
       <c r="F24" s="37"/>
       <c r="G24" s="34"/>
       <c r="H24" s="35"/>
-      <c r="I24" s="69"/>
+      <c r="I24" s="41"/>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="66" t="s">
+      <c r="A25" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="67"/>
-      <c r="C25" s="67"/>
-      <c r="D25" s="67"/>
+      <c r="B25" s="56"/>
+      <c r="C25" s="56"/>
+      <c r="D25" s="56"/>
       <c r="E25" s="21">
         <f>SUM(E18:E24)</f>
         <v>0</v>
@@ -1351,9 +1347,7 @@
       <c r="F25" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="G25" s="70" t="s">
-        <v>24</v>
-      </c>
+      <c r="G25" s="42"/>
       <c r="H25" s="38"/>
       <c r="I25" s="39">
         <f>SUM(I18:I24)</f>
@@ -1362,15 +1356,15 @@
       <c r="J25" s="2"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="64"/>
-      <c r="B26" s="65"/>
-      <c r="C26" s="65"/>
-      <c r="D26" s="65"/>
-      <c r="E26" s="65"/>
-      <c r="F26" s="65"/>
-      <c r="G26" s="65"/>
-      <c r="H26" s="65"/>
-      <c r="I26" s="65"/>
+      <c r="A26" s="53"/>
+      <c r="B26" s="54"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="54"/>
       <c r="J26" s="3"/>
     </row>
     <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1537,17 +1531,17 @@
       <c r="J40" s="6"/>
     </row>
     <row r="41" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="62" t="s">
+      <c r="A41" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B41" s="63"/>
-      <c r="C41" s="63"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="63"/>
-      <c r="F41" s="63"/>
-      <c r="G41" s="63"/>
-      <c r="H41" s="63"/>
-      <c r="I41" s="63"/>
+      <c r="B41" s="52"/>
+      <c r="C41" s="52"/>
+      <c r="D41" s="52"/>
+      <c r="E41" s="52"/>
+      <c r="F41" s="52"/>
+      <c r="G41" s="52"/>
+      <c r="H41" s="52"/>
+      <c r="I41" s="52"/>
       <c r="J41" s="6"/>
     </row>
     <row r="42" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1563,39 +1557,23 @@
       <c r="J42" s="6"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" s="60" t="s">
+      <c r="A43" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="B43" s="61"/>
-      <c r="C43" s="61"/>
-      <c r="D43" s="61"/>
-      <c r="E43" s="61"/>
-      <c r="F43" s="55" t="s">
+      <c r="B43" s="50"/>
+      <c r="C43" s="50"/>
+      <c r="D43" s="50"/>
+      <c r="E43" s="50"/>
+      <c r="F43" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="G43" s="46"/>
-      <c r="H43" s="46"/>
-      <c r="I43" s="46"/>
+      <c r="G43" s="60"/>
+      <c r="H43" s="60"/>
+      <c r="I43" s="60"/>
       <c r="J43" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="G13:I15"/>
-    <mergeCell ref="F43:I43"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="H7:I7"/>
@@ -1612,6 +1590,22 @@
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="G13:I15"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <hyperlinks>

</xml_diff>